<commit_message>
Regenera los análisis temáticos consistentes con los hotspots < 1 ha
Al bajar el umbral a 0,09 ha, se recalcularon los 5 análisis que leen los
hotspots (fragmentación/recurrencia, minería, POMCAS, figuras de protección,
territorios colectivos) y se actualizaron los números derivados en toda la
plataforma y los entregables:

- Minería (títulos+solicitudes): 30,2% -> 40,8% de lo mapeado
- Frentes persistentes (>=3 periodos): 72% -> 78,9% (1.039 -> 1.411 celdas)
- POMCA Río León: 3.860 -> 4.738 ha; parches: 9.107 -> 19.023
- Actualiza hallazgos.json, contenido.ts (aprende), soporte documental
  (metodología), Informe Word y Excel (recalculado, 0 errores)
- AP (12,6%), cuencas y territorios étnicos no cambian (no leen hotspots)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entregables/Dashboard_Deforestacion_CORPOURABA_2000-2024.xlsx
+++ b/entregables/Dashboard_Deforestacion_CORPOURABA_2000-2024.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\drive-download-20260703T192518Z-3-001\observatorio-deforestacion\entregables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88F5E262-0FD7-49BF-BD2B-BF546384204D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0BB4F15-B106-426F-812F-56DC8CFEDA64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -540,7 +540,7 @@
     <t>2019-2023</t>
   </si>
   <si>
-    <t>En 2002-2010 los resguardos indígenas y consejos comunitarios concentraban el 16,4% de la deforestación mapeada; en 2019-2023 concentran el 40,9%. La presión se movió hacia los territorios colectivos mientras el resto de la jurisdicción desacelera.</t>
+    <t>En 2002-2010 los resguardos indígenas y consejos comunitarios concentraban el 16,6% de la deforestación mapeada; en 2019-2023 concentran el 40,6%. La presión se movió hacia los territorios colectivos mientras el resto de la jurisdicción desacelera.</t>
   </si>
   <si>
     <t>dinamica_bosque</t>
@@ -561,7 +561,7 @@
     <t>fragmentacion</t>
   </si>
   <si>
-    <t>72% de la pérdida ocurre en frentes persistentes</t>
+    <t>79% de la pérdida ocurre en frentes persistentes</t>
   </si>
   <si>
     <t>% de ha en celdas recurrentes</t>
@@ -570,7 +570,7 @@
     <t>2002-2023</t>
   </si>
   <si>
-    <t>1.039 celdas de 2×2 km registran deforestación en 3 o más periodos y concentran el 72,2% de las hectáreas deforestadas mapeadas. No son eventos dispersos: son frentes activos y localizables, priorizables para control.</t>
+    <t>1.411 celdas de 2×2 km registran deforestación en 3 o más periodos y concentran el 78,9% de las hectáreas deforestadas mapeadas. No son eventos dispersos: son frentes activos y localizables, priorizables para control.</t>
   </si>
   <si>
     <t>Turbo pierde más bosque; Carepa, la mayor fracción</t>
@@ -624,13 +624,13 @@
     <t>De las 4.513 ha deforestadas en resguardos con medición de área, 3.478 ha corresponden a territorios del pueblo Embera Katío. Los resguardos de Murindó (583 ha), Chaquenodá (558 ha) y Andabú (421 ha) encabezan el ranking.</t>
   </si>
   <si>
-    <t>Frentes activos 10 de 12 periodos en Mutatá y Dabeiba</t>
+    <t>Frentes activos 11 de 12 periodos en Mutatá y Dabeiba</t>
   </si>
   <si>
     <t>periodos con deforestación (máx. observado)</t>
   </si>
   <si>
-    <t>Las celdas más recurrentes de la jurisdicción (piedemonte de Mutatá y Dabeiba, eje de la vía al mar) registran deforestación en 10 de los 12 periodos mapeados, con hasta 127 ha acumuladas por celda de 400 ha. Urrao (179), Turbo (165) y Dabeiba (152) tienen más celdas persistentes.</t>
+    <t>Las celdas más recurrentes de la jurisdicción (piedemonte de Mutatá y Dabeiba, eje de la vía al mar) registran deforestación en 11 de los 12 periodos mapeados, con hasta 136 ha acumuladas por celda de 400 ha. Urrao (249), Turbo (221) y Dabeiba (203) tienen más celdas persistentes.</t>
   </si>
   <si>
     <t>ACIA (Medio Atrato): el territorio colectivo más afectado</t>
@@ -639,13 +639,13 @@
     <t>El Consejo Comunitario Mayor del Medio Atrato acumula 1.255 ha deforestadas, el 55% de la pérdida en consejos comunitarios (2.269 ha). En proporción de su enorme territorio (174.778 ha) es un 0,7%, pero su tendencia acompaña la aceleración del Atrato.</t>
   </si>
   <si>
-    <t>Deforestación atomizada: 9.107 parches, mediana 1,7 ha</t>
+    <t>Deforestación atomizada: 19.023 parches, mediana 1 ha</t>
   </si>
   <si>
-    <t>parches ≥1 ha en 12 periodos</t>
+    <t>parches en 12 periodos (incluye &lt; 1 ha)</t>
   </si>
   <si>
-    <t>El 92% de los parches mide menos de 5 ha (64% del área); solo el 2,5% supera 10 ha pero aporta el 22,5% del área. El tamaño de parche es estable en el tiempo (~2,8 ha): el patrón es de colonización hormiga, no de grandes praderizaciones — con la excepción de Turbo (parche máximo de 738 ha).</t>
+    <t>El 96% de los parches mide menos de 5 ha (70% del área); solo el 1,2% supera 10 ha pero aporta el 19% del área. El tamaño medio de parche es pequeño (~1,6 ha; mediana 0,95 ha) e incluye ahora los focos de menos de 1 ha: el patrón es de colonización hormiga, no de grandes praderizaciones — con la excepción de Turbo (parche máximo de 738 ha).</t>
   </si>
   <si>
     <t>Caribe y Centro desaceleran; Atrato, Nutibara y Urrao aceleran</t>
@@ -810,28 +810,28 @@
     <t>Tule/Guna (Cuna)</t>
   </si>
   <si>
+    <t>Jaikerazavi (Abibe Mutata)</t>
+  </si>
+  <si>
     <t>Rio Chajerado</t>
   </si>
   <si>
     <t>Embera</t>
   </si>
   <si>
-    <t>Jaikerazavi (Abibe Mutata)</t>
+    <t>Pavarando Y Amparrado Medio</t>
   </si>
   <si>
-    <t>Pavarando Y Amparrado Medio</t>
+    <t>Chimurro Y Nendo</t>
   </si>
   <si>
     <t>Chontadural Cañero</t>
   </si>
   <si>
-    <t>Chimurro Y Nendo</t>
+    <t>Polines</t>
   </si>
   <si>
     <t>Sever</t>
-  </si>
-  <si>
-    <t>Polines</t>
   </si>
   <si>
     <t>Amparrado Alto Medio</t>
@@ -846,10 +846,10 @@
     <t>Cañaverales Antado</t>
   </si>
   <si>
-    <t>Rio Jarapeto</t>
+    <t>Jengado Apartado</t>
   </si>
   <si>
-    <t>Jengado Apartado</t>
+    <t>Rio Jarapeto</t>
   </si>
   <si>
     <t>Choromandó Alto y Medio</t>
@@ -876,6 +876,9 @@
     <t>Monzhomando</t>
   </si>
   <si>
+    <t>Narikizavi</t>
+  </si>
+  <si>
     <t>Urada Jiguamiando</t>
   </si>
   <si>
@@ -886,12 +889,6 @@
   </si>
   <si>
     <t>Canime</t>
-  </si>
-  <si>
-    <t>Comunidad Indigena Embera Chami Y Zenu De La Palma</t>
-  </si>
-  <si>
-    <t>Embera Chamí-Zenú</t>
   </si>
   <si>
     <t>Los Almendros (El Bagre)</t>
@@ -909,10 +906,13 @@
     <t>Embera Drua</t>
   </si>
   <si>
-    <t>Rio Bebara</t>
+    <t>Comunidad Indigena Embera Chami Y Zenu De La Palma</t>
   </si>
   <si>
-    <t>Narikizavi</t>
+    <t>Embera Chamí-Zenú</t>
+  </si>
+  <si>
+    <t>Rio Bebara</t>
   </si>
   <si>
     <t>Santa Maria El Charcon</t>
@@ -1419,7 +1419,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-E2DA-44DA-BF62-38CB9459BEEA}"/>
+              <c16:uniqueId val="{00000000-4585-455B-981C-023484993282}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1633,7 +1633,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-853C-4F44-82FB-FEFDE33A469B}"/>
+              <c16:uniqueId val="{00000000-7FD2-4E38-8790-38623504D8E0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1793,7 +1793,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-4E8F-4867-B9BB-A3E023A0EB2E}"/>
+              <c16:uniqueId val="{00000000-8F6E-4391-9E53-D5FFEC099026}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2005,7 +2005,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-FA4E-41E0-B593-D1221F6016B7}"/>
+              <c16:uniqueId val="{00000000-B3C8-487E-ACEF-E5249F2205E4}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2159,7 +2159,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-FA4E-41E0-B593-D1221F6016B7}"/>
+              <c16:uniqueId val="{00000001-B3C8-487E-ACEF-E5249F2205E4}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3052,7 +3052,7 @@
       </c>
       <c r="B24" s="9"/>
       <c r="C24" s="11">
-        <v>3860.1</v>
+        <v>4738.5</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -3061,7 +3061,7 @@
       </c>
       <c r="B25" s="9"/>
       <c r="C25" s="11">
-        <v>2225.1999999999998</v>
+        <v>2739.2</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -3070,7 +3070,7 @@
       </c>
       <c r="B26" s="9"/>
       <c r="C26" s="11">
-        <v>1747.2</v>
+        <v>2368.1999999999998</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -3079,7 +3079,7 @@
       </c>
       <c r="B27" s="9"/>
       <c r="C27" s="11">
-        <v>493.8</v>
+        <v>537.20000000000005</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="B28" s="9"/>
       <c r="C28" s="11">
-        <v>307.2</v>
+        <v>234.2</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -3097,7 +3097,7 @@
       </c>
       <c r="B29" s="9"/>
       <c r="C29" s="11">
-        <v>49.5</v>
+        <v>58.3</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -3106,7 +3106,7 @@
       </c>
       <c r="B30" s="9"/>
       <c r="C30" s="11">
-        <v>41.4</v>
+        <v>42.7</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -3133,7 +3133,7 @@
         <v>250</v>
       </c>
       <c r="C35" s="11">
-        <v>468.3</v>
+        <v>576.6</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -3144,7 +3144,7 @@
         <v>250</v>
       </c>
       <c r="C36" s="11">
-        <v>452.6</v>
+        <v>557.79999999999995</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -3155,7 +3155,7 @@
         <v>250</v>
       </c>
       <c r="C37" s="11">
-        <v>361.6</v>
+        <v>461.6</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -3166,7 +3166,7 @@
         <v>250</v>
       </c>
       <c r="C38" s="11">
-        <v>256.60000000000002</v>
+        <v>312.2</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -3177,7 +3177,7 @@
         <v>250</v>
       </c>
       <c r="C39" s="11">
-        <v>235.9</v>
+        <v>285.2</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -3188,7 +3188,7 @@
         <v>250</v>
       </c>
       <c r="C40" s="11">
-        <v>204.4</v>
+        <v>282.60000000000002</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -3199,7 +3199,7 @@
         <v>257</v>
       </c>
       <c r="C41" s="11">
-        <v>180.8</v>
+        <v>262.10000000000002</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -3207,21 +3207,21 @@
         <v>258</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>259</v>
+        <v>250</v>
       </c>
       <c r="C42" s="11">
-        <v>169.8</v>
+        <v>216.2</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="9" t="s">
+        <v>259</v>
+      </c>
+      <c r="B43" s="9" t="s">
         <v>260</v>
       </c>
-      <c r="B43" s="9" t="s">
-        <v>250</v>
-      </c>
       <c r="C43" s="11">
-        <v>163.1</v>
+        <v>203.8</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -3229,10 +3229,10 @@
         <v>261</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C44" s="11">
-        <v>149.69999999999999</v>
+        <v>184.1</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -3240,10 +3240,10 @@
         <v>262</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>250</v>
+        <v>260</v>
       </c>
       <c r="C45" s="11">
-        <v>145</v>
+        <v>172.6</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
@@ -3251,10 +3251,10 @@
         <v>263</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>259</v>
+        <v>250</v>
       </c>
       <c r="C46" s="11">
-        <v>132.69999999999999</v>
+        <v>165.8</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -3265,7 +3265,7 @@
         <v>250</v>
       </c>
       <c r="C47" s="11">
-        <v>100.2</v>
+        <v>111</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -3276,7 +3276,7 @@
         <v>250</v>
       </c>
       <c r="C48" s="11">
-        <v>75.900000000000006</v>
+        <v>109.9</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -3287,7 +3287,7 @@
         <v>250</v>
       </c>
       <c r="C49" s="11">
-        <v>68</v>
+        <v>95</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -3295,10 +3295,10 @@
         <v>267</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C50" s="11">
-        <v>67.400000000000006</v>
+        <v>82.6</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -3309,7 +3309,7 @@
         <v>250</v>
       </c>
       <c r="C51" s="11">
-        <v>53.4</v>
+        <v>77.099999999999994</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
@@ -3320,7 +3320,7 @@
         <v>250</v>
       </c>
       <c r="C52" s="11">
-        <v>32.5</v>
+        <v>50.2</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
@@ -3328,10 +3328,10 @@
         <v>270</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C53" s="11">
-        <v>27.9</v>
+        <v>32.299999999999997</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
@@ -3339,10 +3339,10 @@
         <v>271</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C54" s="11">
-        <v>22.5</v>
+        <v>32.200000000000003</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
@@ -3353,7 +3353,7 @@
         <v>250</v>
       </c>
       <c r="C55" s="11">
-        <v>19.899999999999999</v>
+        <v>22.2</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
@@ -3361,10 +3361,10 @@
         <v>273</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C56" s="11">
-        <v>14.8</v>
+        <v>19.2</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
@@ -3372,10 +3372,10 @@
         <v>274</v>
       </c>
       <c r="B57" s="9" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C57" s="11">
-        <v>10.1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
@@ -3386,7 +3386,7 @@
         <v>250</v>
       </c>
       <c r="C58" s="11">
-        <v>6.2</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -3397,7 +3397,7 @@
         <v>250</v>
       </c>
       <c r="C59" s="11">
-        <v>5.3</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
@@ -3408,7 +3408,7 @@
         <v>250</v>
       </c>
       <c r="C60" s="11">
-        <v>3.4</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
@@ -3416,10 +3416,10 @@
         <v>278</v>
       </c>
       <c r="B61" s="9" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C61" s="11">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
@@ -3430,7 +3430,7 @@
         <v>250</v>
       </c>
       <c r="C62" s="11">
-        <v>0.4</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
@@ -3438,10 +3438,10 @@
         <v>280</v>
       </c>
       <c r="B63" s="9" t="s">
-        <v>259</v>
+        <v>250</v>
       </c>
       <c r="C63" s="11">
-        <v>0.2</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
@@ -3449,7 +3449,7 @@
         <v>281</v>
       </c>
       <c r="B64" s="9" t="s">
-        <v>282</v>
+        <v>260</v>
       </c>
       <c r="C64" s="11">
         <v>0.1</v>
@@ -3457,13 +3457,13 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="B65" s="9" t="s">
         <v>283</v>
       </c>
-      <c r="B65" s="9" t="s">
-        <v>282</v>
-      </c>
       <c r="C65" s="11">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
@@ -3471,7 +3471,7 @@
         <v>284</v>
       </c>
       <c r="B66" s="9" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C66" s="11">
         <v>0</v>
@@ -3479,10 +3479,10 @@
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="9" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C67" s="11">
         <v>0</v>
@@ -3490,10 +3490,10 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="9" t="s">
+        <v>286</v>
+      </c>
+      <c r="B68" s="9" t="s">
         <v>287</v>
-      </c>
-      <c r="B68" s="9" t="s">
-        <v>288</v>
       </c>
       <c r="C68" s="11">
         <v>0</v>
@@ -3501,10 +3501,10 @@
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="9" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B69" s="9" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C69" s="11">
         <v>0</v>
@@ -3512,7 +3512,7 @@
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="9" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B70" s="9" t="s">
         <v>250</v>
@@ -3523,10 +3523,10 @@
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="9" t="s">
+        <v>290</v>
+      </c>
+      <c r="B71" s="9" t="s">
         <v>291</v>
-      </c>
-      <c r="B71" s="9" t="s">
-        <v>259</v>
       </c>
       <c r="C71" s="11">
         <v>0</v>
@@ -3537,7 +3537,7 @@
         <v>292</v>
       </c>
       <c r="B72" s="9" t="s">
-        <v>250</v>
+        <v>260</v>
       </c>
       <c r="C72" s="11">
         <v>0</v>
@@ -3559,7 +3559,7 @@
         <v>294</v>
       </c>
       <c r="B74" s="9" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C74" s="11">
         <v>0</v>
@@ -3589,7 +3589,7 @@
         <v>297</v>
       </c>
       <c r="C79" s="11">
-        <v>1056.5</v>
+        <v>1334.8</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
@@ -3600,7 +3600,7 @@
         <v>79</v>
       </c>
       <c r="C80" s="11">
-        <v>1022.8</v>
+        <v>1057.2</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
@@ -3611,7 +3611,7 @@
         <v>66</v>
       </c>
       <c r="C81" s="11">
-        <v>303.8</v>
+        <v>360.8</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
@@ -3622,7 +3622,7 @@
         <v>301</v>
       </c>
       <c r="C82" s="11">
-        <v>220.3</v>
+        <v>266.5</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
@@ -3633,7 +3633,7 @@
         <v>79</v>
       </c>
       <c r="C83" s="11">
-        <v>151.80000000000001</v>
+        <v>164.8</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
@@ -3644,7 +3644,7 @@
         <v>79</v>
       </c>
       <c r="C84" s="11">
-        <v>24.4</v>
+        <v>30.2</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
@@ -3655,7 +3655,7 @@
         <v>79</v>
       </c>
       <c r="C85" s="11">
-        <v>13.4</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
@@ -3666,7 +3666,7 @@
         <v>79</v>
       </c>
       <c r="C86" s="11">
-        <v>1.9</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
@@ -67387,7 +67387,7 @@
         <v>165</v>
       </c>
       <c r="C2" s="9">
-        <v>40.9</v>
+        <v>40.6</v>
       </c>
       <c r="D2" s="9" t="s">
         <v>166</v>
@@ -67427,7 +67427,7 @@
         <v>175</v>
       </c>
       <c r="C4" s="9">
-        <v>72.2</v>
+        <v>78.900000000000006</v>
       </c>
       <c r="D4" s="9" t="s">
         <v>176</v>
@@ -67547,7 +67547,7 @@
         <v>196</v>
       </c>
       <c r="C10" s="9">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>197</v>
@@ -67579,7 +67579,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>174</v>
       </c>
@@ -67587,7 +67587,7 @@
         <v>201</v>
       </c>
       <c r="C12" s="9">
-        <v>9107</v>
+        <v>19023</v>
       </c>
       <c r="D12" s="9" t="s">
         <v>202</v>

</xml_diff>

<commit_message>
chore: entregables regenerados y build info actualizados
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entregables/Dashboard_Deforestacion_CORPOURABA_2000-2024.xlsx
+++ b/entregables/Dashboard_Deforestacion_CORPOURABA_2000-2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\drive-download-20260703T192518Z-3-001\observatorio-deforestacion\entregables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0BB4F15-B106-426F-812F-56DC8CFEDA64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23349ECD-0824-462D-9446-757465461408}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Portada" sheetId="1" r:id="rId1"/>
@@ -1256,6 +1256,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:rPr lang="es-CO"/>
               <a:t>Deforestación anualizada (ha/año) — jurisdicción CORPOURABA</a:t>
             </a:r>
           </a:p>
@@ -1471,6 +1472,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
+                  <a:rPr lang="es-CO"/>
                   <a:t>ha/año</a:t>
                 </a:r>
               </a:p>
@@ -1520,6 +1522,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:rPr lang="es-CO"/>
               <a:t>Top 10 municipios por deforestación acumulada (ha)</a:t>
             </a:r>
           </a:p>
@@ -1713,6 +1716,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:rPr lang="es-CO"/>
               <a:t>Distribución por subregión (ha)</a:t>
             </a:r>
           </a:p>
@@ -1842,6 +1846,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:rPr lang="es-CO"/>
               <a:t>Municipio seleccionado vs promedio regional (ha/año)</a:t>
             </a:r>
           </a:p>
@@ -1946,58 +1951,58 @@
                 <c:formatCode>#,##0.0</c:formatCode>
                 <c:ptCount val="18"/>
                 <c:pt idx="0">
-                  <c:v>4.5250000000000004</c:v>
+                  <c:v>1.34</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.4950000000000001</c:v>
+                  <c:v>3.28</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>78.355000000000004</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>41.384999999999998</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>11.77</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>15.925000000000001</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>26.21</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.53</c:v>
+                </c:pt>
+                <c:pt idx="8">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.73499999999999999</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>1.4750000000000001</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>37.22</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>87.29</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>15.25</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>17.09</c:v>
-                </c:pt>
                 <c:pt idx="9">
-                  <c:v>25.12</c:v>
+                  <c:v>3.76</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>35.659999999999997</c:v>
+                  <c:v>16.13</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>4.28</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2.7</c:v>
+                  <c:v>10.53</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1.1200000000000001</c:v>
+                  <c:v>4.92</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0</c:v>
+                  <c:v>40.89</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>5.77</c:v>
+                  <c:v>14.58</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>8.2200000000000006</c:v>
+                  <c:v>58.66</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>12.14</c:v>
+                  <c:v>55.82</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2211,6 +2216,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
+                  <a:rPr lang="es-CO"/>
                   <a:t>ha/año</a:t>
                 </a:r>
               </a:p>
@@ -43570,7 +43576,7 @@
         <v>117</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="G4" s="17" t="s">
         <v>118</v>
@@ -43579,19 +43585,19 @@
     <row r="7" spans="1:11" ht="21" x14ac:dyDescent="0.35">
       <c r="B7" s="19">
         <f>SUM(B11:B28)</f>
-        <v>311.53999999999996</v>
+        <v>537.14</v>
       </c>
       <c r="E7" s="20">
         <f>B7/'Serie regional'!$E$20</f>
-        <v>6.6503691281471523E-3</v>
+        <v>1.1466197834926372E-2</v>
       </c>
       <c r="H7" s="21" t="str">
         <f>INDEX(A11:A28,MATCH(MAX(B11:B28),B11:B28,0))</f>
-        <v>2012-2013</v>
+        <v>2004-2006</v>
       </c>
       <c r="K7" s="21" t="str">
         <f>INDEX(Aux!$B$4:$B$22,MATCH($E$4,Aux!$A$4:$A$22,0))</f>
-        <v>Nutibara</v>
+        <v>Caribe</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -43632,11 +43638,11 @@
       </c>
       <c r="B11" s="11">
         <f>SUMIFS('Serie municipal'!$H$2:$H$1132,'Serie municipal'!$B$2:$B$1132,$E$4,'Serie municipal'!$G$2:$G$1132,"Deforestación",'Serie municipal'!$D$2:$D$1132,$A$11)</f>
-        <v>9.0500000000000007</v>
+        <v>2.68</v>
       </c>
       <c r="C11" s="11">
         <f>B11/'Serie regional'!D2</f>
-        <v>4.5250000000000004</v>
+        <v>1.34</v>
       </c>
       <c r="D11" s="22">
         <f>'Serie regional'!F2</f>
@@ -43654,11 +43660,11 @@
       </c>
       <c r="B12" s="11">
         <f>SUMIFS('Serie municipal'!$H$2:$H$1132,'Serie municipal'!$B$2:$B$1132,$E$4,'Serie municipal'!$G$2:$G$1132,"Deforestación",'Serie municipal'!$D$2:$D$1132,$A$12)</f>
-        <v>8.99</v>
+        <v>6.56</v>
       </c>
       <c r="C12" s="11">
         <f>B12/'Serie regional'!D3</f>
-        <v>4.4950000000000001</v>
+        <v>3.28</v>
       </c>
       <c r="D12" s="22">
         <f>'Serie regional'!F3</f>
@@ -43676,11 +43682,11 @@
       </c>
       <c r="B13" s="11">
         <f>SUMIFS('Serie municipal'!$H$2:$H$1132,'Serie municipal'!$B$2:$B$1132,$E$4,'Serie municipal'!$G$2:$G$1132,"Deforestación",'Serie municipal'!$D$2:$D$1132,$A$13)</f>
-        <v>0</v>
+        <v>156.71</v>
       </c>
       <c r="C13" s="11">
         <f>B13/'Serie regional'!D4</f>
-        <v>0</v>
+        <v>78.355000000000004</v>
       </c>
       <c r="D13" s="22">
         <f>'Serie regional'!F4</f>
@@ -43698,11 +43704,11 @@
       </c>
       <c r="B14" s="11">
         <f>SUMIFS('Serie municipal'!$H$2:$H$1132,'Serie municipal'!$B$2:$B$1132,$E$4,'Serie municipal'!$G$2:$G$1132,"Deforestación",'Serie municipal'!$D$2:$D$1132,$A$14)</f>
-        <v>1.47</v>
+        <v>82.77</v>
       </c>
       <c r="C14" s="11">
         <f>B14/'Serie regional'!D5</f>
-        <v>0.73499999999999999</v>
+        <v>41.384999999999998</v>
       </c>
       <c r="D14" s="22">
         <f>'Serie regional'!F5</f>
@@ -43720,11 +43726,11 @@
       </c>
       <c r="B15" s="11">
         <f>SUMIFS('Serie municipal'!$H$2:$H$1132,'Serie municipal'!$B$2:$B$1132,$E$4,'Serie municipal'!$G$2:$G$1132,"Deforestación",'Serie municipal'!$D$2:$D$1132,$A$15)</f>
-        <v>2.95</v>
+        <v>23.54</v>
       </c>
       <c r="C15" s="11">
         <f>B15/'Serie regional'!D6</f>
-        <v>1.4750000000000001</v>
+        <v>11.77</v>
       </c>
       <c r="D15" s="22">
         <f>'Serie regional'!F6</f>
@@ -43742,11 +43748,11 @@
       </c>
       <c r="B16" s="11">
         <f>SUMIFS('Serie municipal'!$H$2:$H$1132,'Serie municipal'!$B$2:$B$1132,$E$4,'Serie municipal'!$G$2:$G$1132,"Deforestación",'Serie municipal'!$D$2:$D$1132,$A$16)</f>
-        <v>74.44</v>
+        <v>31.85</v>
       </c>
       <c r="C16" s="11">
         <f>B16/'Serie regional'!D7</f>
-        <v>37.22</v>
+        <v>15.925000000000001</v>
       </c>
       <c r="D16" s="22">
         <f>'Serie regional'!F7</f>
@@ -43764,11 +43770,11 @@
       </c>
       <c r="B17" s="11">
         <f>SUMIFS('Serie municipal'!$H$2:$H$1132,'Serie municipal'!$B$2:$B$1132,$E$4,'Serie municipal'!$G$2:$G$1132,"Deforestación",'Serie municipal'!$D$2:$D$1132,$A$17)</f>
-        <v>87.29</v>
+        <v>26.21</v>
       </c>
       <c r="C17" s="11">
         <f>B17/'Serie regional'!D8</f>
-        <v>87.29</v>
+        <v>26.21</v>
       </c>
       <c r="D17" s="22">
         <f>'Serie regional'!F8</f>
@@ -43786,11 +43792,11 @@
       </c>
       <c r="B18" s="11">
         <f>SUMIFS('Serie municipal'!$H$2:$H$1132,'Serie municipal'!$B$2:$B$1132,$E$4,'Serie municipal'!$G$2:$G$1132,"Deforestación",'Serie municipal'!$D$2:$D$1132,$A$18)</f>
-        <v>15.25</v>
+        <v>1.53</v>
       </c>
       <c r="C18" s="11">
         <f>B18/'Serie regional'!D9</f>
-        <v>15.25</v>
+        <v>1.53</v>
       </c>
       <c r="D18" s="22">
         <f>'Serie regional'!F9</f>
@@ -43808,11 +43814,11 @@
       </c>
       <c r="B19" s="11">
         <f>SUMIFS('Serie municipal'!$H$2:$H$1132,'Serie municipal'!$B$2:$B$1132,$E$4,'Serie municipal'!$G$2:$G$1132,"Deforestación",'Serie municipal'!$D$2:$D$1132,$A$19)</f>
-        <v>17.09</v>
+        <v>0</v>
       </c>
       <c r="C19" s="11">
         <f>B19/'Serie regional'!D10</f>
-        <v>17.09</v>
+        <v>0</v>
       </c>
       <c r="D19" s="22">
         <f>'Serie regional'!F10</f>
@@ -43830,11 +43836,11 @@
       </c>
       <c r="B20" s="11">
         <f>SUMIFS('Serie municipal'!$H$2:$H$1132,'Serie municipal'!$B$2:$B$1132,$E$4,'Serie municipal'!$G$2:$G$1132,"Deforestación",'Serie municipal'!$D$2:$D$1132,$A$20)</f>
-        <v>25.12</v>
+        <v>3.76</v>
       </c>
       <c r="C20" s="11">
         <f>B20/'Serie regional'!D11</f>
-        <v>25.12</v>
+        <v>3.76</v>
       </c>
       <c r="D20" s="22">
         <f>'Serie regional'!F11</f>
@@ -43852,11 +43858,11 @@
       </c>
       <c r="B21" s="11">
         <f>SUMIFS('Serie municipal'!$H$2:$H$1132,'Serie municipal'!$B$2:$B$1132,$E$4,'Serie municipal'!$G$2:$G$1132,"Deforestación",'Serie municipal'!$D$2:$D$1132,$A$21)</f>
-        <v>35.659999999999997</v>
+        <v>16.13</v>
       </c>
       <c r="C21" s="11">
         <f>B21/'Serie regional'!D12</f>
-        <v>35.659999999999997</v>
+        <v>16.13</v>
       </c>
       <c r="D21" s="22">
         <f>'Serie regional'!F12</f>
@@ -43874,11 +43880,11 @@
       </c>
       <c r="B22" s="11">
         <f>SUMIFS('Serie municipal'!$H$2:$H$1132,'Serie municipal'!$B$2:$B$1132,$E$4,'Serie municipal'!$G$2:$G$1132,"Deforestación",'Serie municipal'!$D$2:$D$1132,$A$22)</f>
-        <v>4.28</v>
+        <v>0</v>
       </c>
       <c r="C22" s="11">
         <f>B22/'Serie regional'!D13</f>
-        <v>4.28</v>
+        <v>0</v>
       </c>
       <c r="D22" s="22">
         <f>'Serie regional'!F13</f>
@@ -43896,11 +43902,11 @@
       </c>
       <c r="B23" s="11">
         <f>SUMIFS('Serie municipal'!$H$2:$H$1132,'Serie municipal'!$B$2:$B$1132,$E$4,'Serie municipal'!$G$2:$G$1132,"Deforestación",'Serie municipal'!$D$2:$D$1132,$A$23)</f>
-        <v>2.7</v>
+        <v>10.53</v>
       </c>
       <c r="C23" s="11">
         <f>B23/'Serie regional'!D14</f>
-        <v>2.7</v>
+        <v>10.53</v>
       </c>
       <c r="D23" s="22">
         <f>'Serie regional'!F14</f>
@@ -43918,11 +43924,11 @@
       </c>
       <c r="B24" s="11">
         <f>SUMIFS('Serie municipal'!$H$2:$H$1132,'Serie municipal'!$B$2:$B$1132,$E$4,'Serie municipal'!$G$2:$G$1132,"Deforestación",'Serie municipal'!$D$2:$D$1132,$A$24)</f>
-        <v>1.1200000000000001</v>
+        <v>4.92</v>
       </c>
       <c r="C24" s="11">
         <f>B24/'Serie regional'!D15</f>
-        <v>1.1200000000000001</v>
+        <v>4.92</v>
       </c>
       <c r="D24" s="22">
         <f>'Serie regional'!F15</f>
@@ -43940,11 +43946,11 @@
       </c>
       <c r="B25" s="11">
         <f>SUMIFS('Serie municipal'!$H$2:$H$1132,'Serie municipal'!$B$2:$B$1132,$E$4,'Serie municipal'!$G$2:$G$1132,"Deforestación",'Serie municipal'!$D$2:$D$1132,$A$25)</f>
-        <v>0</v>
+        <v>40.89</v>
       </c>
       <c r="C25" s="11">
         <f>B25/'Serie regional'!D16</f>
-        <v>0</v>
+        <v>40.89</v>
       </c>
       <c r="D25" s="22">
         <f>'Serie regional'!F16</f>
@@ -43962,11 +43968,11 @@
       </c>
       <c r="B26" s="11">
         <f>SUMIFS('Serie municipal'!$H$2:$H$1132,'Serie municipal'!$B$2:$B$1132,$E$4,'Serie municipal'!$G$2:$G$1132,"Deforestación",'Serie municipal'!$D$2:$D$1132,$A$26)</f>
-        <v>5.77</v>
+        <v>14.58</v>
       </c>
       <c r="C26" s="11">
         <f>B26/'Serie regional'!D17</f>
-        <v>5.77</v>
+        <v>14.58</v>
       </c>
       <c r="D26" s="22">
         <f>'Serie regional'!F17</f>
@@ -43984,11 +43990,11 @@
       </c>
       <c r="B27" s="11">
         <f>SUMIFS('Serie municipal'!$H$2:$H$1132,'Serie municipal'!$B$2:$B$1132,$E$4,'Serie municipal'!$G$2:$G$1132,"Deforestación",'Serie municipal'!$D$2:$D$1132,$A$27)</f>
-        <v>8.2200000000000006</v>
+        <v>58.66</v>
       </c>
       <c r="C27" s="11">
         <f>B27/'Serie regional'!D18</f>
-        <v>8.2200000000000006</v>
+        <v>58.66</v>
       </c>
       <c r="D27" s="22">
         <f>'Serie regional'!F18</f>
@@ -44006,11 +44012,11 @@
       </c>
       <c r="B28" s="11">
         <f>SUMIFS('Serie municipal'!$H$2:$H$1132,'Serie municipal'!$B$2:$B$1132,$E$4,'Serie municipal'!$G$2:$G$1132,"Deforestación",'Serie municipal'!$D$2:$D$1132,$A$28)</f>
-        <v>12.14</v>
+        <v>55.82</v>
       </c>
       <c r="C28" s="11">
         <f>B28/'Serie regional'!D19</f>
-        <v>12.14</v>
+        <v>55.82</v>
       </c>
       <c r="D28" s="22">
         <f>'Serie regional'!F19</f>

</xml_diff>